<commit_message>
Update Gantt chart template for improved project timeline visualization
Replaced the existing Gantt chart template file (`attached_assets/gantt_template.xlsx`) with an updated version.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/210b8442-4fe8-4b47-9541-b0d29770d286/57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170/TXtvpM0
</commit_message>
<xml_diff>
--- a/attached_assets/gantt_template.xlsx
+++ b/attached_assets/gantt_template.xlsx
@@ -13198,7 +13198,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:E200"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="55.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13222,7 +13228,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2. Enter Start Date in column C - Excel will show a calendar picker</v>
+        <v>2. Enter Start Date in column C - see "DATE ENTRY METHODS" below for calendar options</v>
       </c>
     </row>
     <row r="6">
@@ -13247,42 +13253,42 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TASK ORGANIZATION</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>• PHASE headers organize major project phases (Outline Level 1)</v>
+        <v>DATE ENTRY METHODS - CHOOSE YOUR PREFERRED OPTION</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>• PACKAGE headers organize vendor categories (Outline Level 1)</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>• Individual tasks under each package (Outline Level 2)</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>OPTION 1: KEYBOARD ENTRY (Built-in, Works Everywhere)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>PHASES INCLUDED</v>
+        <v>• Click any date cell and type: 2024-01-15 (YYYY-MM-DD format)</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>1. Design &amp; Approvals - Initial design phase with client approvals</v>
+        <v>• Or press Ctrl+; to insert today's date</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2. Vendor Evaluation → Quotes → Finalisation → Work Orders</v>
+        <v>• Simple and fast for experienced users</v>
       </c>
     </row>
     <row r="18">
@@ -13292,468 +13298,1154 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>PACKAGES INCLUDED</v>
+        <v>OPTION 2: VISUAL CALENDAR PICKER - RECOMMENDED ⭐</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>• Civil, Electricals, Plumbing, Kitchens, Bathrooms, Audio, Automation</v>
+        <v>For the best experience, install a free calendar add-in:</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>• Lighting, HVAC, Curtains, Furniture, Wardrobes, Flooring, Painting</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>• False Ceiling, Mirrors, Soft Furnishings, Décor, Upholstery, Storage</v>
+        <v>METHOD A: Randy's Date Picker (Works in Excel 2016/2019/2021/365, 32-bit &amp; 64-bit)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>• Each package follows the same workflow:</v>
+        <v>Step 1: Download the add-in</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  1. Vendor Evaluation → 2. Meetings/Survey → 3. RFQs → 4. Quotes</v>
+        <v xml:space="preserve">        • Google search: "Randy Austin date picker Excel download"</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  5. Comparison → 6. Finalisation → 7. Work Order</v>
+        <v xml:space="preserve">        • Or visit: https://bettersolutions.com/excel/date-picker/ (trusted source)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v xml:space="preserve">        • Download the .xlam file (Excel add-in)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>AUTOMATIC DATE CALCULATION</v>
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>• When you enter Start Date + Duration, Finish Date calculates automatically</v>
+        <v>Step 2: Install the add-in</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>• Formula: Finish = Start + Duration - 1 day</v>
+        <v xml:space="preserve">        • Open Excel</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>• Example: Start = Jan 1, Duration = 5 → Finish = Jan 5</v>
+        <v xml:space="preserve">        • File → Options → Add-ins</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>• Works for both actual dates and target dates</v>
+        <v xml:space="preserve">        • At bottom, select "Excel Add-ins" → Click "Go..."</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
+        <v xml:space="preserve">        • Click "Browse..." → Find your downloaded .xlam file</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>DATE ENTRY WITH CALENDAR</v>
+        <v xml:space="preserve">        • Check the box next to "Randy's Date Picker" → Click OK</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>• Click any Start or Finish date cell</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>• Excel shows a calendar icon or date picker</v>
+        <v>Step 3: Use the calendar</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>• Select date from calendar or type YYYY-MM-DD (e.g., 2024-01-15)</v>
+        <v xml:space="preserve">        • Click any date cell in your template</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v/>
+        <v xml:space="preserve">        • A floating calendar popup appears automatically</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>COLUMN REFERENCE</v>
+        <v xml:space="preserve">        • Click a date to insert it</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Column</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Description</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Notes</v>
+        <v xml:space="preserve">        • Works for all date columns (no configuration needed)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Task identifier (1-249)</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Pre-filled, do not change</v>
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Name</v>
-      </c>
-      <c r="B41" t="str">
-        <v>Task name</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Pre-filled with your project tasks</v>
+        <v>METHOD B: Kutools Date Picker (Commercial, Full-Featured)</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Start</v>
-      </c>
-      <c r="B42" t="str">
-        <v>Start date (CALENDAR PICKER)</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Click for calendar, auto-calculates finish</v>
+        <v xml:space="preserve">        • Visit: https://www.extendoffice.com/product/kutools-for-excel.html</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Finish</v>
-      </c>
-      <c r="B43" t="str">
-        <v>End date (AUTO-CALCULATED)</v>
-      </c>
-      <c r="C43" t="str">
-        <v>Auto: Start + Duration - 1</v>
+        <v xml:space="preserve">        • Free trial available, then $49 for permanent license</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Duration</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Working days</v>
-      </c>
-      <c r="C44" t="str">
-        <v>Pre-filled, adjust as needed</v>
+        <v xml:space="preserve">        • Includes 300+ Excel tools beyond just date picking</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>% Complete</v>
-      </c>
-      <c r="B45" t="str">
-        <v>Progress (0-100)</v>
-      </c>
-      <c r="C45" t="str">
-        <v>Update as work progresses</v>
+        <v xml:space="preserve">        • Calendar appears when clicking any date cell</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Predecessors</v>
-      </c>
-      <c r="B46" t="str">
-        <v>Dependencies</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Pre-configured: TaskID(Type)</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Resource Names</v>
-      </c>
-      <c r="B47" t="str">
-        <v>Assigned team</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Pre-filled: Designer, Client, Vendor, etc.</v>
+        <v>METHOD C: Built-in ActiveX Control (Legacy, 32-bit Excel Only)</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Status</v>
-      </c>
-      <c r="B48" t="str">
-        <v>Current status</v>
-      </c>
-      <c r="C48" t="str">
-        <v>not_started, in_progress, completed, blocked</v>
+        <v xml:space="preserve">        ⚠️ Not recommended - doesn't work in 64-bit Excel</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Priority</v>
-      </c>
-      <c r="B49" t="str">
-        <v>Task priority</v>
-      </c>
-      <c r="C49" t="str">
-        <v>low, medium, high (auto-set for key tasks)</v>
+        <v xml:space="preserve">        • Enable Developer tab: File → Options → Customize Ribbon → Check "Developer"</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Approval Required</v>
-      </c>
-      <c r="B50" t="str">
-        <v>Needs approval? (Y/N)</v>
-      </c>
-      <c r="C50" t="str">
-        <v>Pre-set for approval tasks</v>
+        <v xml:space="preserve">        • Developer → Insert → More Controls</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Materials</v>
-      </c>
-      <c r="B51" t="str">
-        <v>Required materials</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Optional</v>
+        <v xml:space="preserve">        • Select "Microsoft Date and Time Picker Control 6.0"</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Owner</v>
-      </c>
-      <c r="B52" t="str">
-        <v>Task owner</v>
-      </c>
-      <c r="C52" t="str">
-        <v>Optional</v>
+        <v xml:space="preserve">        • Manually link to each cell (time-consuming for 249 tasks)</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Target Start</v>
-      </c>
-      <c r="B53" t="str">
-        <v>Planned start (CALENDAR)</v>
-      </c>
-      <c r="C53" t="str">
-        <v>Optional planning dates</v>
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Target Finish</v>
-      </c>
-      <c r="B54" t="str">
-        <v>Planned finish (AUTO-CALC)</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Auto: Target Start + Duration - 1</v>
+        <v>COMPARISON: Which Method Should You Choose?</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Remarks</v>
+        <v>Method</v>
       </c>
       <c r="B55" t="str">
-        <v>Notes</v>
+        <v>Ease of Use</v>
       </c>
       <c r="C55" t="str">
-        <v>Pre-filled with milestones</v>
+        <v>64-bit Compatible</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Cost</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Recommendation</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Outline Level</v>
+        <v>Keyboard Entry</v>
       </c>
       <c r="B56" t="str">
-        <v>Hierarchy (1 or 2)</v>
+        <v>Easy</v>
       </c>
       <c r="C56" t="str">
-        <v>1=Phase/Package, 2=Task</v>
+        <v>Yes</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Free</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Good for quick edits</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Color</v>
+        <v>Randy's Picker</v>
       </c>
       <c r="B57" t="str">
-        <v>Task color</v>
+        <v>Very Easy</v>
       </c>
       <c r="C57" t="str">
-        <v>Optional hex code: #4A90E2</v>
+        <v>Yes</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Free</v>
+      </c>
+      <c r="E57" t="str">
+        <v>⭐ BEST for most users</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v/>
+        <v>Kutools</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Very Easy</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D58" t="str">
+        <v>$49</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Best for power users</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>DEPENDENCY TYPES</v>
+        <v>ActiveX Control</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Difficult</v>
+      </c>
+      <c r="C59" t="str">
+        <v>No</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Free</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Avoid - outdated</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Format</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Meaning</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Example</v>
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>TaskID(FS)</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Finish-to-Start (most common)</v>
-      </c>
-      <c r="C61" t="str">
-        <v>2(FS) = Task 2 finishes before this starts</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>TaskID(SS)</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Start-to-Start</v>
-      </c>
-      <c r="C62" t="str">
-        <v>3(SS) = Task 3 starts before this starts</v>
+        <v>TASK ORGANIZATION</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>TaskID(FF)</v>
-      </c>
-      <c r="B63" t="str">
-        <v>Finish-to-Finish</v>
-      </c>
-      <c r="C63" t="str">
-        <v>4(FF) = Task 4 finishes before this finishes</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>TaskID(SF)</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Start-to-Finish (rare)</v>
-      </c>
-      <c r="C64" t="str">
-        <v>5(SF) = Task 5 starts before this finishes</v>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>With lag</v>
-      </c>
-      <c r="B65" t="str">
-        <v>Add delay</v>
-      </c>
-      <c r="C65" t="str">
-        <v>2(FS)+3 = Wait 3 days after Task 2 finishes</v>
+        <v>PHASES INCLUDED</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Multiple</v>
-      </c>
-      <c r="B66" t="str">
-        <v>Comma-separated</v>
-      </c>
-      <c r="C66" t="str">
-        <v>4(FS),5(FS) = Wait for both 4 and 5</v>
+        <v>1. Design &amp; Approvals - Initial design phase with client approvals</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v/>
+        <v>2. Vendor Evaluation → Quotes → Finalisation → Work Orders</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>PRE-CONFIGURED DEPENDENCIES</v>
+        <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>All task dependencies are pre-configured based on typical project workflow</v>
+        <v>PACKAGES INCLUDED (20 Categories)</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Each package follows sequential steps with dependencies on previous steps</v>
+        <v>• Civil, Electricals, Plumbing, Kitchens, Bathrooms, Audio, Automation</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Cross-package dependencies link packages to design phase completion</v>
+        <v>• Lighting, HVAC, Curtains, Furniture, Wardrobes, Flooring, Painting</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v/>
+        <v>• False Ceiling, Mirrors, Soft Furnishings, Décor, Upholstery, Storage</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>CRITICAL PATH ANALYSIS</v>
+        <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>After importing, the system will:</v>
+        <v>Each package follows the same 7-step workflow:</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>• Calculate Early Start (ES) and Early Finish (EF) for all tasks</v>
+        <v xml:space="preserve">  1. Vendor Evaluation (shortlist) → 2. Vendor Meetings / Site Survey</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>• Calculate Late Start (LS) and Late Finish (LF) for all tasks</v>
+        <v xml:space="preserve">  3. RFQs Issued → 4. Quotes Received &amp; Clarifications</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>• Identify critical tasks (zero float - must complete on time)</v>
+        <v xml:space="preserve">  5. Quote Comparison &amp; Negotiation → 6. Vendor Finalisation</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>• Show total project duration and critical path percentage</v>
+        <v xml:space="preserve">  7. Work Order / PO Release</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>• Detect circular dependencies and prevent import errors</v>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>HIERARCHY</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>• PHASE headers: Outline Level 1 (major project phases)</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>• PACKAGE headers: Outline Level 1 (vendor categories)</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>• Individual tasks: Outline Level 2 (specific activities)</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>AUTOMATIC DATE CALCULATIONS</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>• When you enter Start Date + Duration, Finish Date calculates automatically</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>• Formula: Finish = Start + Duration - 1 day</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>• Example: Start = Jan 1, Duration = 5 → Finish = Jan 5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>• Works for both Actual dates (C, D) and Target dates (N, O)</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>• You can override auto-calculated dates if needed</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>COLUMN REFERENCE (18 Columns)</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Description</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Task identifier (1-249)</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Pre-filled, do not change</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Task name</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Pre-filled with your project tasks</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Start</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Start date</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Use calendar picker or type YYYY-MM-DD</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Finish</v>
+      </c>
+      <c r="B103" t="str">
+        <v>End date (AUTO-CALC)</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Auto: Start + Duration - 1, can override</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Duration</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Working days</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Pre-filled, adjust as needed</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>% Complete</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Progress (0-100)</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Update as work progresses</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Predecessors</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Dependencies</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Pre-configured: TaskID(Type)</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Resource Names</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Assigned team</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Designer, Client, Vendor, etc.</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Current status</v>
+      </c>
+      <c r="C108" t="str">
+        <v>not_started, in_progress, completed, blocked</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Priority</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Task priority</v>
+      </c>
+      <c r="C109" t="str">
+        <v>low, medium, high (auto-set for key tasks)</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Approval Required</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Needs approval? (Y/N)</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Pre-set for approval tasks</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Materials</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Required materials</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Optional - add as needed</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Task owner name</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Optional - assign task owner</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Target Start</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Planned start</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Optional planning dates</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Target Finish</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Planned finish (AUTO-CALC)</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Auto: Target Start + Duration - 1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Remarks</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Milestones and special notes</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Outline Level</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Hierarchy (1 or 2)</v>
+      </c>
+      <c r="C116" t="str">
+        <v>1=Phase/Package, 2=Task</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Color</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Task color</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Optional hex code: #4A90E2</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>DEPENDENCY TYPES (Critical Path Analysis)</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Format</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Meaning</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Example</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>TaskID(FS)</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Finish-to-Start</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Task finishes before this starts</v>
+      </c>
+      <c r="D124" t="str">
+        <v>2(FS) = Wait for Task 2 to finish</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>TaskID(SS)</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Start-to-Start</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Task starts before this starts</v>
+      </c>
+      <c r="D125" t="str">
+        <v>3(SS) = Wait for Task 3 to start</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>TaskID(FF)</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Finish-to-Finish</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Task finishes before this finishes</v>
+      </c>
+      <c r="D126" t="str">
+        <v>4(FF) = Must finish with Task 4</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>TaskID(SF)</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Start-to-Finish</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Task starts before this finishes</v>
+      </c>
+      <c r="D127" t="str">
+        <v>5(SF) = Rare, special cases</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>With lag</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Add delay</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Wait extra days after dependency</v>
+      </c>
+      <c r="D128" t="str">
+        <v>2(FS)+3 = 3 days after Task 2</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Multiple</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Comma-separated</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Wait for multiple tasks</v>
+      </c>
+      <c r="D129" t="str">
+        <v>4(FS),5(FS) = Wait for both</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>PRE-CONFIGURED DEPENDENCIES</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>All task dependencies are pre-configured based on typical interior design workflow:</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>• Design phase tasks flow sequentially (Client Brief → Schematics → Working Drawings)</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>• Each package starts after Client Sign-off on drawings</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>• Within each package, tasks follow the 7-step workflow sequentially</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>• You can modify dependencies if your project workflow differs</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>CRITICAL PATH ANALYSIS (After Importing to PixelCraft Designer)</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>After importing this template into PixelCraft Designer, the system will:</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>✓ Calculate Early Start (ES) and Early Finish (EF) for all tasks</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>✓ Calculate Late Start (LS) and Late Finish (LF) for all tasks</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>✓ Identify critical tasks (zero float - must complete on time)</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>✓ Show total project duration in working days</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>✓ Display critical path percentage (% of tasks on critical path)</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>✓ Detect circular dependencies and prevent import errors</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>✓ Highlight critical tasks with visual badges</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>WHAT IS THE CRITICAL PATH?</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>The critical path is the longest sequence of dependent tasks that determines</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>the minimum project duration. Any delay in critical path tasks delays the</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>entire project. Tasks not on the critical path have "float" (slack time).</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>KEY METRICS:</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>• Total Float: How many days a task can be delayed without affecting project end</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>• Critical Tasks: Tasks with zero float (must complete on schedule)</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>• Project Duration: Earliest possible project completion date</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>TIPS FOR BEST RESULTS</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>1. Install Randy's Date Picker first for easiest date entry</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>2. Start by filling in Start dates for the first few tasks</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>3. Let the Finish dates auto-calculate (they use the formula)</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>4. Adjust Duration values based on your project needs</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>5. Review pre-configured dependencies - modify if your workflow differs</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>6. Use Status column to track progress: not_started → in_progress → completed</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>7. Set Priority to "high" for time-sensitive or client-facing tasks</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>8. Import into PixelCraft Designer to see Critical Path Analysis</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>9. Download updated schedule from PixelCraft to get latest progress</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>10. Keep Approval Required tasks visible - they often become bottlenecks</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>TROUBLESHOOTING</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Problem: Date validation message appears but no calendar</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Solution: You need to install a calendar add-in (see OPTION 2 above)</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>Problem: Finish date not calculating automatically</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Solution: Make sure Start date AND Duration are both filled in</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>Problem: Import fails with "circular dependency" error</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>Solution: Check Predecessors column - a task cannot depend on itself or</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v xml:space="preserve">         create a loop (e.g., Task 5 → Task 10 → Task 5)</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>Problem: Critical path shows 100% of tasks as critical</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>Solution: Dependencies may be too strict - some packages could start in</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v xml:space="preserve">         parallel instead of sequentially</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Problem: Excel shows "####" in date columns</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Solution: Column is too narrow - double-click column border to auto-fit</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>For support with PixelCraft Designer system, contact your administrator</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E200"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gantt chart template to improve project timeline visualization
Replaces the existing Gantt chart template with an updated version.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/210b8442-4fe8-4b47-9541-b0d29770d286/57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170/mvtaV32
</commit_message>
<xml_diff>
--- a/attached_assets/gantt_template.xlsx
+++ b/attached_assets/gantt_template.xlsx
@@ -400,6 +400,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R250"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1" hidden="true"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1" hidden="true"/>
+    <col min="12" max="12" width="25.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="30.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="10.83203125" customWidth="1" hidden="true"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13199,12 +13219,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E200"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
Update Gantt chart template for project timeline visualization
Replaced the existing Gantt chart template Excel file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/210b8442-4fe8-4b47-9541-b0d29770d286/57bb8da2-c3cb-4c56-8f00-0f1b8c9d0170/mvtaV32
</commit_message>
<xml_diff>
--- a/attached_assets/gantt_template.xlsx
+++ b/attached_assets/gantt_template.xlsx
@@ -401,24 +401,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R250"/>
   <cols>
-    <col min="1" max="1" width="6.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1" hidden="true"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1" hidden="true"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="30.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="10.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1"/>
+    <col min="2" max="2"/>
+    <col min="3" max="3"/>
+    <col min="4" max="4"/>
+    <col min="5" max="5"/>
+    <col min="6" max="6"/>
+    <col min="7" max="7"/>
+    <col min="8" max="8"/>
+    <col min="9" max="9"/>
+    <col min="10" max="10"/>
+    <col min="11" max="11"/>
+    <col min="12" max="12"/>
+    <col min="13" max="13"/>
+    <col min="14" max="14"/>
+    <col min="15" max="15"/>
+    <col min="16" max="16"/>
+    <col min="17" max="17"/>
+    <col min="18" max="18"/>
+    <col min="19" max="19" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>